<commit_message>
Add edge-detail view and fix explorer edge rendering
- Taxi (circuit-board) edge routing; bundled-bezier fan for edges that
  share a node pair so bidirectional links no longer stack and garble.
- Aggregate relationships per direction (one labeled edge, with a count
  when a direction carries several) to avoid 32-arc hairballs.
- Canonicalize relationship targets in the parser so the stale
  310 - WH Enrollment name resolves to 310 - Enrollment Intake instead
  of stubbing a phantom Lookup; add the name alias.
- Edge click opens an edge-detail side panel listing every individual
  relationship (name, via-field, match-field, pull count) with source
  and target navigation and a selected-edge glow. Workflow edges stay
  non-interactive. Document the three side-panel view categories.
</commit_message>
<xml_diff>
--- a/output/global/cross-workspace-inventory.xlsx
+++ b/output/global/cross-workspace-inventory.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllForms'!$A$3:$E$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllForms'!$A$3:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$G$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>2296</v>
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>310 - WH Enrollment</t>
+          <t>Climate Zones</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -998,33 +998,8 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>socal-whp</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Climate Zones</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Lookup</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>(no JSON)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:E14"/>
+  <autoFilter ref="A3:E13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add FieldAssignments generator (Excel/CSV), ingest sce-be re-export
- scripts/expand_field_assignments.py: mass-generate a WFEngine
  workflow's top-level FieldAssignments from an Excel or CSV mapping
  (source field / assignment type / Resolution field). Standard header
  labels matched by name; three-column files with custom headers fall
  back to positional order. Field names validated against
  docs/field-index.json; dry-run default, --apply writes.
- Scoped to Constant/FromTrigger: Expression and Clear/Set Null have no
  confirmed platform ValueType string anywhere in data/, so rows using
  them are hard errors (tracked under TODO Candidates).
- Verified against the real sce-be 'Update Existing Measures' workflow
  and the BE210 mapping CSV (37/41 rows resolve; 4 flagged legitimately).
- data/sce-be: fresh platform re-export (+4 workflows, 111 -> 115
  fleet-wide); all views regenerated.
- 12 new unit tests; CLAUDE.md/README.md/TODO.md updated.
</commit_message>
<xml_diff>
--- a/output/global/cross-workspace-inventory.xlsx
+++ b/output/global/cross-workspace-inventory.xlsx
@@ -20,10 +20,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllForms'!$A$3:$F$318</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$J$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$J$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'FormNameCollisions'!$A$3:$D$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DuplicateFlows'!$A$3:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'WorkflowReuse'!$A$3:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'WorkflowReuse'!$A$3:$I$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'FormFamilies'!$A$3:$F$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FieldTemplates'!$A$3:$D$2755</definedName>
   </definedNames>
@@ -764,7 +764,7 @@
         <v>36</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -9149,7 +9149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10709,17 +10709,17 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>210_ENROLLMENT_APPROVED</t>
+          <t>210_REQUIRES_CORRECTIONS</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Approved</t>
+          <t>Requires Corrections</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status is 'Enrollment Approved'.</t>
+          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -10755,17 +10755,17 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>210_REQUIRES_CORRECTIONS</t>
+          <t>255_INSTALLATION_DESKTOP</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Requires Corrections</t>
+          <t>Installation Desktop Review</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status is 'Corrections Required'.</t>
+          <t>Runs when a 255 - BE Installation Form record is updated, and only if Submission Status is 'Ready for Review'.</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -10780,7 +10780,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>210 - Enrollment &amp; Assessment Form</t>
+          <t>255 - BE Installation Form</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr">
@@ -10801,17 +10801,17 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>255_INSTALLATION_DESKTOP</t>
+          <t>255_INSTALLATION</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Installation Desktop Review</t>
+          <t>Installation Approved</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 255 - BE Installation Form record is updated, and only if Submission Status is 'Ready for Review'.</t>
+          <t>Runs when a 255 - BE Installation Form record is updated, and only if Review Status is 'Approved'.</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -10847,17 +10847,17 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>255_INSTALLATION</t>
+          <t>255_INSTALLATION_2</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Installation Approved</t>
+          <t>Installation Requires Corrections</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 255 - BE Installation Form record is updated, and only if Review Status is 'Approved'.</t>
+          <t>Runs when a 255 - BE Installation Form record is updated, and only if Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -10893,17 +10893,17 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>255_INSTALLATION_2</t>
+          <t>INVOICE_INVOICE_SUBMITTED_BY</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Installation Requires Corrections</t>
+          <t>Invoice Submitted by Contractor - Final</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 255 - BE Installation Form record is updated, and only if Review Status is 'Corrections Required'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Number (Final) compares to 'None'.</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>255 - BE Installation Form</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H40" s="9" t="inlineStr">
@@ -10939,17 +10939,17 @@
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_INVOICE_SUBMITTED_BY</t>
+          <t>INVOICE_INVOICE_SUBMITTED_BY_2</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Invoice Submitted by Contractor - Final</t>
+          <t>Invoice Submitted by Contractor - Down Payment</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Number (Final) compares to 'None'.</t>
+          <t>Runs when a new Invoice record is created, and only if Request Down Payment is 'True'.</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -10969,7 +10969,7 @@
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="I41" s="9" t="inlineStr"/>
@@ -10985,17 +10985,17 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_INVOICE_SUBMITTED_BY_2</t>
+          <t>INVOICE_APPROVED_BY</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Invoice Submitted by Contractor - Down Payment</t>
+          <t>Approved by Coordinator - Down Payment</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Runs when a new Invoice record is created, and only if Request Down Payment is 'True'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Pending Review by PM' and Request Down Payment is 'True'.</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
@@ -11015,7 +11015,7 @@
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>Create</t>
+          <t>Update</t>
         </is>
       </c>
       <c r="I42" s="9" t="inlineStr"/>
@@ -11031,17 +11031,17 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_APPROVED_BY</t>
+          <t>INVOICE_CORRECTIONS_REQUIRED</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Approved by Coordinator - Down Payment</t>
+          <t>Corrections Required - Down Payment</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Pending Review by PM' and Request Down Payment is 'True'.</t>
+          <t>Runs when a Invoice record is updated, and only if Request Down Payment is 'True' and Invoice Status (DP) compares to 'Pending Corrections'.</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
@@ -11077,17 +11077,17 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_CORRECTIONS_REQUIRED</t>
+          <t>INVOICE_INVOICE_REJECTED_BY</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Corrections Required - Down Payment</t>
+          <t>Invoice Rejected by Management - Final</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Request Down Payment is 'True' and Invoice Status (DP) compares to 'Pending Corrections'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Rejected' and Invoice Number (Final) compares to 'None' and Assigned User (Final) is 'Jose Landeros'.</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -11123,17 +11123,17 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_INVOICE_REJECTED_BY</t>
+          <t>INVOICE_CORRECTIONS_REQUIRED_2</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Invoice Rejected by Management - Final</t>
+          <t>Corrections Required - Final</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Rejected' and Invoice Number (Final) compares to 'None' and Assigned User (Final) is 'Jose Landeros'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) compares to 'Pending Corrections'.</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
@@ -11169,17 +11169,17 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_CORRECTIONS_REQUIRED_2</t>
+          <t>210_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Corrections Required - Final</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) compares to 'Pending Corrections'.</t>
+          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status compares to 'Pending Review' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr">
@@ -11215,7 +11215,7 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>210_REVIEW_NOTIFICATION</t>
+          <t>255_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -11225,7 +11225,7 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status compares to 'Pending Review' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a 255 - BE Installation Form record is updated, and only if Installation Status compares to 'Draft' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
@@ -11240,7 +11240,7 @@
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>210 - Enrollment &amp; Assessment Form</t>
+          <t>255 - BE Installation Form</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>255_REVIEW_NOTIFICATION</t>
+          <t>INVOICE_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 255 - BE Installation Form record is updated, and only if Installation Status compares to 'Draft' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) compares to 'None' and Processor Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>255 - BE Installation Form</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H48" s="9" t="inlineStr">
@@ -11307,17 +11307,17 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_REVIEW_NOTIFICATION</t>
+          <t>210_UPDATE_RECORDS</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Update Records</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) compares to 'None' and Processor Name compares to 'None'.</t>
+          <t>Runs when a new 210 - Enrollment &amp; Assessment Form record is created.</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -11332,12 +11332,12 @@
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="I49" s="9" t="inlineStr"/>
@@ -11348,22 +11348,22 @@
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>sdge-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>410_DESKTOP_REVIEW</t>
+          <t>255_UPDATE_RECORDS</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Desktop Review</t>
+          <t>Update Records</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 410 - WH Enrollment record is updated, and only if Submission Status is 'Completed &amp; Ready for Review'.</t>
+          <t>Runs when a new 255 - BE Installation Form record is created, and only if Enrollment Number compares to 'None'.</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
@@ -11378,12 +11378,12 @@
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment</t>
+          <t>255 - BE Installation Form</t>
         </is>
       </c>
       <c r="H50" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="I50" s="9" t="inlineStr"/>
@@ -11394,12 +11394,12 @@
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>sdge-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>410_ENROLLMENT_APPROVED</t>
+          <t>210_ENROLLMENT_APPROVED</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 410 - WH Enrollment record is updated, and only if Review Status is 'Enrollment Approved'.</t>
+          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status is 'Enrollment Approved'.</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="H51" s="9" t="inlineStr">
@@ -11440,22 +11440,22 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>sdge-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>410_ENROLLMENT</t>
+          <t>200_CREATE_ENROLLMENT</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Corrections Required</t>
+          <t>Create Enrollment Form</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 410 - WH Enrollment record is updated, and only if Review Status is 'Corrections Required'.</t>
+          <t>Runs when a new 200 - Account record is created, and only if Lead Status is 'Completed Lead' and Project Stage is 'Enrollment' and Project Status is 'In Progress'.</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -11470,38 +11470,42 @@
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment</t>
+          <t>200 - Account</t>
         </is>
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
-        </is>
-      </c>
-      <c r="I52" s="9" t="inlineStr"/>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
       <c r="J52" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>sdge-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>415_DESKTOP_REVIEW</t>
+          <t>210_UPDATE_EXISTING</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Desktop Review</t>
+          <t>Update Existing Measures</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Submission Status is 'Ready for Review'.</t>
+          <t>Runs when a 210 - Enrollment &amp; Assessment Form record is updated, and only if MAROMA Review Status is 'Enrollment Approved' and Enrollment Approved Date is not '2026-07-01T00:00:00-07:00'.</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -11516,7 +11520,7 @@
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="H53" s="9" t="inlineStr">
@@ -11524,9 +11528,13 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I53" s="9" t="inlineStr"/>
+      <c r="I53" s="9" t="inlineStr">
+        <is>
+          <t>255 - BE Installation Form</t>
+        </is>
+      </c>
       <c r="J53" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="22" customHeight="1">
@@ -11537,17 +11545,17 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>415_ASSESSMENT_APPROVED</t>
+          <t>410_DESKTOP_REVIEW</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Assessment Approved</t>
+          <t>Desktop Review</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Review Status compares to 'Assessment Approved'.</t>
+          <t>Runs when a 410 - WH Enrollment record is updated, and only if Submission Status is 'Completed &amp; Ready for Review'.</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -11562,7 +11570,7 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment</t>
+          <t>410 - WH Enrollment</t>
         </is>
       </c>
       <c r="H54" s="9" t="inlineStr">
@@ -11583,17 +11591,17 @@
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>415_ASSESSMENT_REQUIRES</t>
+          <t>410_ENROLLMENT_APPROVED</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Assessment Requires Corrections</t>
+          <t>Enrollment Approved</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Review Status is 'Corrections Required'.</t>
+          <t>Runs when a 410 - WH Enrollment record is updated, and only if Review Status is 'Enrollment Approved'.</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
@@ -11608,7 +11616,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment</t>
+          <t>410 - WH Enrollment</t>
         </is>
       </c>
       <c r="H55" s="9" t="inlineStr">
@@ -11629,17 +11637,17 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>425_INSTALLATION_READY</t>
+          <t>410_ENROLLMENT</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Installation Ready for Review</t>
+          <t>Enrollment Corrections Required</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 425 - San Diego Installation record is updated, and only if Submission Status is 'Ready for Review'.</t>
+          <t>Runs when a 410 - WH Enrollment record is updated, and only if Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
@@ -11654,7 +11662,7 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>425 - San Diego Installation</t>
+          <t>410 - WH Enrollment</t>
         </is>
       </c>
       <c r="H56" s="9" t="inlineStr">
@@ -11675,17 +11683,17 @@
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>425_INSTALLATION</t>
+          <t>415_DESKTOP_REVIEW</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Installation Approved</t>
+          <t>Desktop Review</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 425 - San Diego Installation record is updated, and only if Review Status is 'Approved'.</t>
+          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Submission Status is 'Ready for Review'.</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
@@ -11700,7 +11708,7 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>425 - San Diego Installation</t>
+          <t>415 - San Diego WHP Assessment</t>
         </is>
       </c>
       <c r="H57" s="9" t="inlineStr">
@@ -11721,17 +11729,17 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>425_INSTALLATION_2</t>
+          <t>415_ASSESSMENT_APPROVED</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Installation Rejected</t>
+          <t>Assessment Approved</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 425 - San Diego Installation record is updated, and only if Review Status is 'Corrections Required'.</t>
+          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Review Status compares to 'Assessment Approved'.</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
@@ -11746,7 +11754,7 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>425 - San Diego Installation</t>
+          <t>415 - San Diego WHP Assessment</t>
         </is>
       </c>
       <c r="H58" s="9" t="inlineStr">
@@ -11767,17 +11775,17 @@
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_INVOICE</t>
+          <t>415_ASSESSMENT_REQUIRES</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Final Invoice Pending Corrections</t>
+          <t>Assessment Requires Corrections</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Review Status (Coordinator) is 'Pending Corrections' or Review Status (PM) is 'Pending Corrections' or Review Status (Management) is 'Pending Corrections' or Invoice Status compares to 'Pending Corrections'.</t>
+          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
@@ -11792,7 +11800,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>415 - San Diego WHP Assessment</t>
         </is>
       </c>
       <c r="H59" s="9" t="inlineStr">
@@ -11813,17 +11821,17 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_APPROVED_BY</t>
+          <t>425_INSTALLATION_READY</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Final Approved by Coordinator</t>
+          <t>Installation Ready for Review</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status compares to 'Pending Review by PM' or Review Status (Coordinator) compares to 'Approved'.</t>
+          <t>Runs when a 425 - San Diego Installation record is updated, and only if Submission Status is 'Ready for Review'.</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
@@ -11838,7 +11846,7 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>425 - San Diego Installation</t>
         </is>
       </c>
       <c r="H60" s="9" t="inlineStr">
@@ -11859,17 +11867,17 @@
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_APPROVED_FOR</t>
+          <t>425_INSTALLATION</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Final Approved for Payment</t>
+          <t>Installation Approved</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status is 'Approved for Final Payment' or Review Status (Management) is 'Approved'.</t>
+          <t>Runs when a 425 - San Diego Installation record is updated, and only if Review Status is 'Approved'.</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
@@ -11884,7 +11892,7 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>425 - San Diego Installation</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
@@ -11905,17 +11913,17 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>ACCOUNT_CONTRACTOR_SUBMITS</t>
+          <t>425_INSTALLATION_2</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Contractor Submits Final Invoice</t>
+          <t>Installation Rejected</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Account Management (400) record is updated, and only if Submit Invoice is 'True'.</t>
+          <t>Runs when a 425 - San Diego Installation record is updated, and only if Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
@@ -11930,7 +11938,7 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400)</t>
+          <t>425 - San Diego Installation</t>
         </is>
       </c>
       <c r="H62" s="9" t="inlineStr">
@@ -11938,13 +11946,9 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I62" s="9" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
+      <c r="I62" s="9" t="inlineStr"/>
       <c r="J62" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" ht="22" customHeight="1">
@@ -11955,17 +11959,17 @@
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>ACCOUNT_CONTRACTOR_SUBMITS_2</t>
+          <t>INVOICE_FINAL_INVOICE</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Contractor Submits Invoice Revision</t>
+          <t>Final Invoice Pending Corrections</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Account Management (400) record is updated, and only if Final Invoice Amount compares to 'None' or Final Invoice Number compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Review Status (Coordinator) is 'Pending Corrections' or Review Status (PM) is 'Pending Corrections' or Review Status (Management) is 'Pending Corrections' or Invoice Status compares to 'Pending Corrections'.</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
@@ -11980,7 +11984,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400)</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H63" s="9" t="inlineStr">
@@ -12001,17 +12005,17 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>ACCOUNT_CUSTOMER_INTEREST</t>
+          <t>INVOICE_FINAL_APPROVED_BY</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Customer Interest Receipt</t>
+          <t>Final Approved by Coordinator</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Account Management (400) record is updated, and only if Send Email Confirmation Receipt is 'True'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status compares to 'Pending Review by PM' or Review Status (Coordinator) compares to 'Approved'.</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
@@ -12026,7 +12030,7 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400)</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H64" s="9" t="inlineStr">
@@ -12047,17 +12051,17 @@
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>410_REVIEW_NOTIFICATION</t>
+          <t>INVOICE_FINAL_APPROVED_FOR</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Final Approved for Payment</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 410 - WH Enrollment record is updated, and only if Submission Status is 'None' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status is 'Approved for Final Payment' or Review Status (Management) is 'Approved'.</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -12072,7 +12076,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H65" s="9" t="inlineStr">
@@ -12093,17 +12097,17 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>415_REVIEW_NOTIFICATION</t>
+          <t>ACCOUNT_CONTRACTOR_SUBMITS</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Contractor Submits Final Invoice</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Assessment Status compares to 'Draft' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a Account Management (400) record is updated, and only if Submit Invoice is 'True'.</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
@@ -12118,7 +12122,7 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment</t>
+          <t>Account Management (400)</t>
         </is>
       </c>
       <c r="H66" s="9" t="inlineStr">
@@ -12126,9 +12130,13 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I66" s="9" t="inlineStr"/>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
       <c r="J66" s="9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" ht="22" customHeight="1">
@@ -12139,17 +12147,17 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>425_REVIEW_NOTIFICATION</t>
+          <t>ACCOUNT_CONTRACTOR_SUBMITS_2</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Contractor Submits Invoice Revision</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 425 - San Diego Installation record is updated, and only if Installation Status compares to 'None' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a Account Management (400) record is updated, and only if Final Invoice Amount compares to 'None' or Final Invoice Number compares to 'None'.</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
@@ -12164,7 +12172,7 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>425 - San Diego Installation</t>
+          <t>Account Management (400)</t>
         </is>
       </c>
       <c r="H67" s="9" t="inlineStr">
@@ -12185,17 +12193,17 @@
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_REVIEW_NOTIFICATION</t>
+          <t>ACCOUNT_CUSTOMER_INTEREST</t>
         </is>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Customer Interest Receipt</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status compares to 'None' and Processor Name compares to 'None'.</t>
+          <t>Runs when a Account Management (400) record is updated, and only if Send Email Confirmation Receipt is 'True'.</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
@@ -12210,7 +12218,7 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Account Management (400)</t>
         </is>
       </c>
       <c r="H68" s="9" t="inlineStr">
@@ -12231,17 +12239,17 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>ACCOUNT_APPROVED_FOR_INSTALL</t>
+          <t>410_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Approved for Install</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Account Management (400) record is updated, and only if Project Stage is 'Installation' and Project Status is 'In Progress' and Assessment Status is 'Approved for Install'.</t>
+          <t>Runs when a 410 - WH Enrollment record is updated, and only if Submission Status is 'None' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
@@ -12256,7 +12264,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400)</t>
+          <t>410 - WH Enrollment</t>
         </is>
       </c>
       <c r="H69" s="9" t="inlineStr">
@@ -12277,17 +12285,17 @@
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>410_UPDATE_ACCOUNT</t>
+          <t>415_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Update Account Status from Enrollment 410</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 410 - WH Enrollment record is updated, and only if Submission Status compares to 'None'.</t>
+          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Assessment Status compares to 'Draft' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
@@ -12302,7 +12310,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment</t>
+          <t>415 - San Diego WHP Assessment</t>
         </is>
       </c>
       <c r="H70" s="9" t="inlineStr">
@@ -12310,13 +12318,9 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I70" s="9" t="inlineStr">
-        <is>
-          <t>Account Management (400)</t>
-        </is>
-      </c>
+      <c r="I70" s="9" t="inlineStr"/>
       <c r="J70" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" ht="22" customHeight="1">
@@ -12327,17 +12331,17 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>415_UPDATE_ACCOUNT</t>
+          <t>425_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Update Account Status from Assessment Form 415</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Review Status compares to 'None'.</t>
+          <t>Runs when a 425 - San Diego Installation record is updated, and only if Installation Status compares to 'None' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
@@ -12352,7 +12356,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment</t>
+          <t>425 - San Diego Installation</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
@@ -12360,13 +12364,9 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I71" s="9" t="inlineStr">
-        <is>
-          <t>Account Management (400)</t>
-        </is>
-      </c>
+      <c r="I71" s="9" t="inlineStr"/>
       <c r="J71" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1">
@@ -12377,17 +12377,17 @@
       </c>
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>ACCOUNT_REFRESH_ACCOUNT</t>
+          <t>INVOICE_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Refresh Account</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Runs on a schedule (every Friday at 20:00), checking Account Management (400) records.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status compares to 'None' and Processor Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
@@ -12402,12 +12402,12 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400)</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
         <is>
-          <t>Create</t>
+          <t>Update</t>
         </is>
       </c>
       <c r="I72" s="9" t="inlineStr"/>
@@ -12418,22 +12418,22 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sdge-whp</t>
         </is>
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>310_DESKTOP_REVIEW</t>
+          <t>ACCOUNT_APPROVED_FOR_INSTALL</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Desktop Review</t>
+          <t>Approved for Install</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Enrollment Status is 'Pending Review'.</t>
+          <t>Runs when a Account Management (400) record is updated, and only if Project Stage is 'Installation' and Project Status is 'In Progress' and Assessment Status is 'Approved for Install'.</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
@@ -12448,7 +12448,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>Account Management (400)</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -12464,22 +12464,22 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sdge-whp</t>
         </is>
       </c>
       <c r="B74" s="9" t="inlineStr">
         <is>
-          <t>310_ENROLLMENT_APPROVED</t>
+          <t>410_UPDATE_ACCOUNT</t>
         </is>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Approved</t>
+          <t>Update Account Status from Enrollment 410</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Review Status is 'Enrollment Approved'.</t>
+          <t>Runs when a 410 - WH Enrollment record is updated, and only if Submission Status compares to 'None'.</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
@@ -12494,7 +12494,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>410 - WH Enrollment</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -12502,30 +12502,34 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I74" s="9" t="inlineStr"/>
+      <c r="I74" s="9" t="inlineStr">
+        <is>
+          <t>Account Management (400)</t>
+        </is>
+      </c>
       <c r="J74" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sdge-whp</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
         <is>
-          <t>310_ENROLLMENT</t>
+          <t>415_UPDATE_ACCOUNT</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Corrections Required</t>
+          <t>Update Account Status from Assessment Form 415</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Review Status is 'Corrections Required'.</t>
+          <t>Runs when a 415 - San Diego WHP Assessment record is updated, and only if Review Status compares to 'None'.</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
@@ -12540,7 +12544,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>415 - San Diego WHP Assessment</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -12548,30 +12552,34 @@
           <t>Update</t>
         </is>
       </c>
-      <c r="I75" s="9" t="inlineStr"/>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>Account Management (400)</t>
+        </is>
+      </c>
       <c r="J75" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sdge-whp</t>
         </is>
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
-          <t>315_DESKTOP_REVIEW</t>
+          <t>ACCOUNT_REFRESH_ACCOUNT</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Desktop Review</t>
+          <t>Refresh Account</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Submission Status is 'Ready for Review'.</t>
+          <t>Runs on a schedule (every Friday at 20:00), checking Account Management (400) records.</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
@@ -12586,12 +12594,12 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>315 - SoCal WHP Assessment</t>
+          <t>Account Management (400)</t>
         </is>
       </c>
       <c r="H76" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="I76" s="9" t="inlineStr"/>
@@ -12607,17 +12615,17 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>315_APPROVED</t>
+          <t>310_DESKTOP_REVIEW</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Desktop Review</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Review Status is 'Assessment Approved'.</t>
+          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Enrollment Status is 'Pending Review'.</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
@@ -12632,7 +12640,7 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>315 - SoCal WHP Assessment</t>
+          <t>310 - Enrollment Intake</t>
         </is>
       </c>
       <c r="H77" s="9" t="inlineStr">
@@ -12653,17 +12661,17 @@
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>315_SUBMISSION_RESULTS</t>
+          <t>310_ENROLLMENT_APPROVED</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Submission Results</t>
+          <t>Enrollment Approved</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Assessment Status compares to 'Corrections Required' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Review Status is 'Enrollment Approved'.</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
@@ -12678,7 +12686,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>315 - SoCal WHP Assessment</t>
+          <t>310 - Enrollment Intake</t>
         </is>
       </c>
       <c r="H78" s="9" t="inlineStr">
@@ -12699,17 +12707,17 @@
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>300_CUSTOMER_INTEREST</t>
+          <t>310_ENROLLMENT</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Customer Interest Receipt</t>
+          <t>Enrollment Corrections Required</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Send Email Confirmation Receipt is 'True'.</t>
+          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
@@ -12724,7 +12732,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>310 - Enrollment Intake</t>
         </is>
       </c>
       <c r="H79" s="9" t="inlineStr">
@@ -12745,17 +12753,17 @@
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>325_READY_FOR_REVIEW</t>
+          <t>315_DESKTOP_REVIEW</t>
         </is>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>Ready for Review</t>
+          <t>Desktop Review</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 325 - SoCal Installation record is updated, and only if Installation Status is 'Pending Review'.</t>
+          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Submission Status is 'Ready for Review'.</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
@@ -12770,7 +12778,7 @@
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>325 - SoCal Installation</t>
+          <t>315 - SoCal WHP Assessment</t>
         </is>
       </c>
       <c r="H80" s="9" t="inlineStr">
@@ -12791,17 +12799,17 @@
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
-          <t>325_INSTALLATION</t>
+          <t>315_APPROVED</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>Installation Rejected</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 325 - SoCal Installation record is updated, and only if Review Status is 'Corrections Required'.</t>
+          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Review Status is 'Assessment Approved'.</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
@@ -12816,7 +12824,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>325 - SoCal Installation</t>
+          <t>315 - SoCal WHP Assessment</t>
         </is>
       </c>
       <c r="H81" s="9" t="inlineStr">
@@ -12837,17 +12845,17 @@
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>395_INSPECTION_RESULT</t>
+          <t>315_SUBMISSION_RESULTS</t>
         </is>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>Inspection Result</t>
+          <t>Submission Results</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Status compares to 'None' and Post-Inspection Status is at least 'Open'.</t>
+          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Assessment Status compares to 'Corrections Required' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
@@ -12862,7 +12870,7 @@
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>315 - SoCal WHP Assessment</t>
         </is>
       </c>
       <c r="H82" s="9" t="inlineStr">
@@ -12883,17 +12891,17 @@
       </c>
       <c r="B83" s="9" t="inlineStr">
         <is>
-          <t>395_WORK_ORDER_ASSIGNED</t>
+          <t>300_CUSTOMER_INTEREST</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>Work Order Assigned to Inspector User</t>
+          <t>Customer Interest Receipt</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Employee compares to 'None'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if Send Email Confirmation Receipt is 'True'.</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
@@ -12908,7 +12916,7 @@
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="H83" s="9" t="inlineStr">
@@ -12929,17 +12937,17 @@
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>300_HANDOFF_TO</t>
+          <t>325_READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>Handoff to Installation Contractor</t>
+          <t>Ready for Review</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Dispatch to Installation Contractor is 'True' and Primary Contractor is at least '06b924d0-99ae-a554-1893-3a12bf2fd6a8'.</t>
+          <t>Runs when a 325 - SoCal Installation record is updated, and only if Installation Status is 'Pending Review'.</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
@@ -12954,7 +12962,7 @@
       </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>325 - SoCal Installation</t>
         </is>
       </c>
       <c r="H84" s="9" t="inlineStr">
@@ -12975,17 +12983,17 @@
       </c>
       <c r="B85" s="9" t="inlineStr">
         <is>
-          <t>300_CONTRACTOR</t>
+          <t>325_INSTALLATION</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>Contractor Requesting Down Payment</t>
+          <t>Installation Rejected</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if DP Invoice Received Date compares to '2025-05-14T07:20:00-07:00' or Down Payment Invoice Number compares to 'None' and Request Down Payment is 'True' and Submit Final Invoice is 'None'.</t>
+          <t>Runs when a 325 - SoCal Installation record is updated, and only if Review Status is 'Corrections Required'.</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
@@ -13000,7 +13008,7 @@
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>325 - SoCal Installation</t>
         </is>
       </c>
       <c r="H85" s="9" t="inlineStr">
@@ -13021,17 +13029,17 @@
       </c>
       <c r="B86" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_DP_APPROVED_BY</t>
+          <t>395_INSPECTION_RESULT</t>
         </is>
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>DP Approved by Coordinator</t>
+          <t>Inspection Result</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Pending Review by PM' or Coordinator Review Status (DP) is 'Approved'.</t>
+          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Status compares to 'None' and Post-Inspection Status is at least 'Open'.</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
@@ -13046,7 +13054,7 @@
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>395 - Inspection Work Order</t>
         </is>
       </c>
       <c r="H86" s="9" t="inlineStr">
@@ -13067,17 +13075,17 @@
       </c>
       <c r="B87" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_DP_CORRECTIONS</t>
+          <t>395_WORK_ORDER_ASSIGNED</t>
         </is>
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>DP Corrections Required</t>
+          <t>Work Order Assigned to Inspector User</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Coordinator Review Status (DP) is 'Corrections Required' or PM Review Status (DP) is 'Corrections Required' and Down Payment is 'True' and Review Status (DP) is 'Corrections Required' and Invoice Status Note (DP) compares to 'Rejected'.</t>
+          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Employee compares to 'None'.</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
@@ -13092,7 +13100,7 @@
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>395 - Inspection Work Order</t>
         </is>
       </c>
       <c r="H87" s="9" t="inlineStr">
@@ -13113,17 +13121,17 @@
       </c>
       <c r="B88" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_DP_APPROVED_BY_2</t>
+          <t>300_HANDOFF_TO</t>
         </is>
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>DP Approved by Program Manager</t>
+          <t>Handoff to Installation Contractor</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Approved for Down Payment' and Down Payment is 'True' and Received Invoice Date (Final) compares to '2025-05-27T15:30:00-07:00'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if Dispatch to Installation Contractor is 'True' and Primary Contractor is at least '06b924d0-99ae-a554-1893-3a12bf2fd6a8'.</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
@@ -13138,7 +13146,7 @@
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="H88" s="9" t="inlineStr">
@@ -13159,17 +13167,17 @@
       </c>
       <c r="B89" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_INVOICE</t>
+          <t>300_CONTRACTOR</t>
         </is>
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>Final Invoice Rejected by Management</t>
+          <t>Contractor Requesting Down Payment</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Installation Invoice is 'True' and Review Status - Management (Final) is 'Rejected'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if DP Invoice Received Date compares to '2025-05-14T07:20:00-07:00' or Down Payment Invoice Number compares to 'None' and Request Down Payment is 'True' and Submit Final Invoice is 'None'.</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
@@ -13184,7 +13192,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="H89" s="9" t="inlineStr">
@@ -13205,17 +13213,17 @@
       </c>
       <c r="B90" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_APPROVED_BY</t>
+          <t>INVOICE_DP_APPROVED_BY</t>
         </is>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>Final Approved by Coordinator</t>
+          <t>DP Approved by Coordinator</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) is 'Pending Review by PM' or Review Status - Coordinator (Final) is 'Approved'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Pending Review by PM' or Coordinator Review Status (DP) is 'Approved'.</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
@@ -13251,17 +13259,17 @@
       </c>
       <c r="B91" s="9" t="inlineStr">
         <is>
-          <t>300_CONTRACTOR_SUBMITS</t>
+          <t>INVOICE_DP_CORRECTIONS</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>Contractor Submits Final Invoice</t>
+          <t>DP Corrections Required</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Final Invoice Amount compares to 'None' or Final Invoice Number compares to 'None' and Submit Final Invoice is 'True'.</t>
+          <t>Runs when a Invoice record is updated, and only if Coordinator Review Status (DP) is 'Corrections Required' or PM Review Status (DP) is 'Corrections Required' and Down Payment is 'True' and Review Status (DP) is 'Corrections Required' and Invoice Status Note (DP) compares to 'Rejected'.</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
@@ -13276,7 +13284,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H91" s="9" t="inlineStr">
@@ -13297,17 +13305,17 @@
       </c>
       <c r="B92" s="9" t="inlineStr">
         <is>
-          <t>395_UPDATED_NOTE_TO</t>
+          <t>INVOICE_DP_APPROVED_BY_2</t>
         </is>
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>Updated Note to Inspector</t>
+          <t>DP Approved by Program Manager</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Notes compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (DP) is 'Approved for Down Payment' and Down Payment is 'True' and Received Invoice Date (Final) compares to '2025-05-27T15:30:00-07:00'.</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
@@ -13322,7 +13330,7 @@
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H92" s="9" t="inlineStr">
@@ -13343,17 +13351,17 @@
       </c>
       <c r="B93" s="9" t="inlineStr">
         <is>
-          <t>395_UPDATED_NOTE_BY</t>
+          <t>INVOICE_FINAL_INVOICE</t>
         </is>
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>Updated Note by MAROMA</t>
+          <t>Final Invoice Rejected by Management</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Notes compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Installation Invoice is 'True' and Review Status - Management (Final) is 'Rejected'.</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
@@ -13368,7 +13376,7 @@
       </c>
       <c r="G93" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H93" s="9" t="inlineStr">
@@ -13389,17 +13397,17 @@
       </c>
       <c r="B94" s="9" t="inlineStr">
         <is>
-          <t>300_CONTRACTOR_SUBMITS_2</t>
+          <t>INVOICE_FINAL_APPROVED_BY</t>
         </is>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>Contractor Submits Enrollment Invoice</t>
+          <t>Final Approved by Coordinator</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Invoice Enrollment is 'True' and Enrollment Invoice Amount compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) is 'Pending Review by PM' or Review Status - Coordinator (Final) is 'Approved'.</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
@@ -13414,7 +13422,7 @@
       </c>
       <c r="G94" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H94" s="9" t="inlineStr">
@@ -13435,17 +13443,17 @@
       </c>
       <c r="B95" s="9" t="inlineStr">
         <is>
-          <t>300_CONTRACTOR_2</t>
+          <t>300_CONTRACTOR_SUBMITS</t>
         </is>
       </c>
       <c r="C95" s="9" t="inlineStr">
         <is>
-          <t>Contractor Requesting Down Payment - Initial</t>
+          <t>Contractor Submits Final Invoice</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Request Down Payment is 'True' and DP Invoice Received Date compares to '2025-05-20T09:36:00-07:00' and Submit Final Invoice is 'None'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if Final Invoice Amount compares to 'None' or Final Invoice Number compares to 'None' and Submit Final Invoice is 'True'.</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
@@ -13481,17 +13489,17 @@
       </c>
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_ENROLLMENT_INVOICE</t>
+          <t>395_UPDATED_NOTE_TO</t>
         </is>
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Invoice Approved for Payment</t>
+          <t>Updated Note to Inspector</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Management Review Status (Enrollment) compares to 'Approved' and Assigned User (Enrollment) is 'Julie Blanco'.</t>
+          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Notes compares to 'None'.</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
@@ -13506,7 +13514,7 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>395 - Inspection Work Order</t>
         </is>
       </c>
       <c r="H96" s="9" t="inlineStr">
@@ -13527,17 +13535,17 @@
       </c>
       <c r="B97" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_ENROLLMENT_INVOICE_2</t>
+          <t>395_UPDATED_NOTE_BY</t>
         </is>
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Invoice Rejected by Management</t>
+          <t>Updated Note by MAROMA</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Management Review Status (Enrollment) is 'Rejected' and Invoice Status Note (Enrollment) compares to 'None'.</t>
+          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Notes compares to 'None'.</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
@@ -13552,7 +13560,7 @@
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>395 - Inspection Work Order</t>
         </is>
       </c>
       <c r="H97" s="9" t="inlineStr">
@@ -13573,17 +13581,17 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_ENROLLMENT_INVOICE_3</t>
+          <t>300_CONTRACTOR_SUBMITS_2</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Invoice Rejected by PM</t>
+          <t>Contractor Submits Enrollment Invoice</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Review Status - Management (Final) is 'Rejected'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if Invoice Enrollment is 'True' and Enrollment Invoice Amount compares to 'None'.</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
@@ -13598,7 +13606,7 @@
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="H98" s="9" t="inlineStr">
@@ -13619,17 +13627,17 @@
       </c>
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>395_UPDATED_NOTE</t>
+          <t>300_CONTRACTOR_2</t>
         </is>
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>Updated Note</t>
+          <t>Contractor Requesting Down Payment - Initial</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Note compares to 'None'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if Request Down Payment is 'True' and DP Invoice Received Date compares to '2025-05-20T09:36:00-07:00' and Submit Final Invoice is 'None'.</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
@@ -13644,7 +13652,7 @@
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="H99" s="9" t="inlineStr">
@@ -13665,17 +13673,17 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>395_RE_INSPECTION_STATUS</t>
+          <t>INVOICE_ENROLLMENT_INVOICE</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>Re-Inspection Status Change</t>
+          <t>Enrollment Invoice Approved for Payment</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Status compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Management Review Status (Enrollment) compares to 'Approved' and Assigned User (Enrollment) is 'Julie Blanco'.</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
@@ -13690,7 +13698,7 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H100" s="9" t="inlineStr">
@@ -13711,17 +13719,17 @@
       </c>
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_INVOICE_2</t>
+          <t>INVOICE_ENROLLMENT_INVOICE_2</t>
         </is>
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>Final Invoice Rejected by PM</t>
+          <t>Enrollment Invoice Rejected by Management</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Installation Invoice is 'True' and Review Status - PM (Final) is 'Rejected'.</t>
+          <t>Runs when a Invoice record is updated, and only if Management Review Status (Enrollment) is 'Rejected' and Invoice Status Note (Enrollment) compares to 'None'.</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
@@ -13757,17 +13765,17 @@
       </c>
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_DP_INVOICE_REJECTED</t>
+          <t>INVOICE_ENROLLMENT_INVOICE_3</t>
         </is>
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>DP Invoice Rejected by PM</t>
+          <t>Enrollment Invoice Rejected by PM</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Down Payment is 'True' and PM Review Status (DP) is 'Rejected'.</t>
+          <t>Runs when a Invoice record is updated, and only if Review Status - Management (Final) is 'Rejected'.</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
@@ -13803,17 +13811,17 @@
       </c>
       <c r="B103" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_CORRECTIONS</t>
+          <t>395_UPDATED_NOTE</t>
         </is>
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>Final Corrections Required</t>
+          <t>Updated Note</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Review Status - Coordinator (Final) is 'Pending Corrections' or Review Status - PM (Final) is 'Pending Corrections' or Review Status - Management (Final) is 'Pending Corrections' and Invoice Status Note (Final) compares to 'None' and Invoice Status (Final) is 'Pending Corrections'.</t>
+          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Note compares to 'None'.</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
@@ -13828,7 +13836,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>395 - Inspection Work Order</t>
         </is>
       </c>
       <c r="H103" s="9" t="inlineStr">
@@ -13849,17 +13857,17 @@
       </c>
       <c r="B104" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_ENROLLMENT_INVOICE_4</t>
+          <t>395_RE_INSPECTION_STATUS</t>
         </is>
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>Enrollment Invoice Corrections Required</t>
+          <t>Re-Inspection Status Change</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Coordinator Review Status (Enrollment) is 'Corrections Required' or Management Review Status (Enrollment) is 'Corrections Required' or PM Review Status (Enrollment) is 'Corrections Required' and Invoice Status Note (Enrollment) compares to 'None'.</t>
+          <t>Runs when a 395 - Inspection Work Order record is updated, and only if Inspection Status compares to 'None'.</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
@@ -13874,7 +13882,7 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>395 - Inspection Work Order</t>
         </is>
       </c>
       <c r="H104" s="9" t="inlineStr">
@@ -13895,17 +13903,17 @@
       </c>
       <c r="B105" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_CREATE_CUSTOMER</t>
+          <t>INVOICE_FINAL_INVOICE_2</t>
         </is>
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>Create Customer Backup</t>
+          <t>Final Invoice Rejected by PM</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Review Status - Management (Final) is 'Approved'.</t>
+          <t>Runs when a Invoice record is updated, and only if Installation Invoice is 'True' and Review Status - PM (Final) is 'Rejected'.</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
@@ -13941,17 +13949,17 @@
       </c>
       <c r="B106" s="9" t="inlineStr">
         <is>
-          <t>310_NOTIFY_ELITE_DESERT</t>
+          <t>INVOICE_DP_INVOICE_REJECTED</t>
         </is>
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>Notify Elite Desert Plumbing for Apex Approval</t>
+          <t>DP Invoice Rejected by PM</t>
         </is>
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Review Status compares to 'Approved' or Enrollment Status compares to 'Approved' and Primary Contractor is '90ba06f0-3ef0-a013-6316-3a1bfa9772bf'.</t>
+          <t>Runs when a Invoice record is updated, and only if Down Payment is 'True' and PM Review Status (DP) is 'Rejected'.</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
@@ -13966,7 +13974,7 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H106" s="9" t="inlineStr">
@@ -13987,17 +13995,17 @@
       </c>
       <c r="B107" s="9" t="inlineStr">
         <is>
-          <t>300_APPROVED_FOR_INSTALL</t>
+          <t>INVOICE_FINAL_CORRECTIONS</t>
         </is>
       </c>
       <c r="C107" s="9" t="inlineStr">
         <is>
-          <t>Approved for Install</t>
+          <t>Final Corrections Required</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Project Stage is 'Installation' and Project Status is 'In Progress' and Assessment Status is 'Approved for Install'.</t>
+          <t>Runs when a Invoice record is updated, and only if Review Status - Coordinator (Final) is 'Pending Corrections' or Review Status - PM (Final) is 'Pending Corrections' or Review Status - Management (Final) is 'Pending Corrections' and Invoice Status Note (Final) compares to 'None' and Invoice Status (Final) is 'Pending Corrections'.</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
@@ -14012,7 +14020,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H107" s="9" t="inlineStr">
@@ -14033,17 +14041,17 @@
       </c>
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>310_REVIEW_NOTIFICATION</t>
+          <t>INVOICE_ENROLLMENT_INVOICE_4</t>
         </is>
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Enrollment Invoice Corrections Required</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Enrollment Status compares to 'None' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Coordinator Review Status (Enrollment) is 'Corrections Required' or Management Review Status (Enrollment) is 'Corrections Required' or PM Review Status (Enrollment) is 'Corrections Required' and Invoice Status Note (Enrollment) compares to 'None'.</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
@@ -14058,7 +14066,7 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H108" s="9" t="inlineStr">
@@ -14079,17 +14087,17 @@
       </c>
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>315_REVIEW_NOTIFICATION</t>
+          <t>INVOICE_CREATE_CUSTOMER</t>
         </is>
       </c>
       <c r="C109" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Create Customer Backup</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Assessment Status compares to 'None' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a Invoice record is updated, and only if Review Status - Management (Final) is 'Approved'.</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
@@ -14104,7 +14112,7 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>315 - SoCal WHP Assessment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="H109" s="9" t="inlineStr">
@@ -14125,17 +14133,17 @@
       </c>
       <c r="B110" s="9" t="inlineStr">
         <is>
-          <t>325_REVIEW_NOTIFICATION</t>
+          <t>310_NOTIFY_ELITE_DESERT</t>
         </is>
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Notify Elite Desert Plumbing for Apex Approval</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 325 - SoCal Installation record is updated, and only if Installation Status compares to 'None' and Reviewer Name compares to 'None'.</t>
+          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Review Status compares to 'Approved' or Enrollment Status compares to 'Approved' and Primary Contractor is '90ba06f0-3ef0-a013-6316-3a1bfa9772bf'.</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
@@ -14150,7 +14158,7 @@
       </c>
       <c r="G110" s="9" t="inlineStr">
         <is>
-          <t>325 - SoCal Installation</t>
+          <t>310 - Enrollment Intake</t>
         </is>
       </c>
       <c r="H110" s="9" t="inlineStr">
@@ -14171,17 +14179,17 @@
       </c>
       <c r="B111" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_REVIEW_NOTIFICATION</t>
+          <t>300_APPROVED_FOR_INSTALL</t>
         </is>
       </c>
       <c r="C111" s="9" t="inlineStr">
         <is>
-          <t>Review Notification (Operations)</t>
+          <t>Approved for Install</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) compares to 'None' and Processor Name (Final) compares to 'None' and Invoice Status (Final) is at least 'Pending Review'.</t>
+          <t>Runs when a 300 - Account Management record is updated, and only if Project Stage is 'Installation' and Project Status is 'In Progress' and Assessment Status is 'Approved for Install'.</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
@@ -14196,7 +14204,7 @@
       </c>
       <c r="G111" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="H111" s="9" t="inlineStr">
@@ -14217,17 +14225,17 @@
       </c>
       <c r="B112" s="9" t="inlineStr">
         <is>
-          <t>300_CONTRACTOR_SUBMITS_3</t>
+          <t>310_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C112" s="9" t="inlineStr">
         <is>
-          <t>Contractor Submits Assessment Invoice</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is updated, and only if Invoice Assessment is 'True' and Assessment Invoice Amount compares to 'None'.</t>
+          <t>Runs when a 310 - Enrollment Intake record is updated, and only if Enrollment Status compares to 'None' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
@@ -14242,7 +14250,7 @@
       </c>
       <c r="G112" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>310 - Enrollment Intake</t>
         </is>
       </c>
       <c r="H112" s="9" t="inlineStr">
@@ -14263,17 +14271,17 @@
       </c>
       <c r="B113" s="9" t="inlineStr">
         <is>
-          <t>INVOICE_FINAL_APPROVED_FOR</t>
+          <t>315_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C113" s="9" t="inlineStr">
         <is>
-          <t>Final Approved for Payment</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) is 'Approved for Final Payment' and Review Status - Management (Final) is 'Approved'.</t>
+          <t>Runs when a 315 - SoCal WHP Assessment record is updated, and only if Assessment Status compares to 'None' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
@@ -14288,7 +14296,7 @@
       </c>
       <c r="G113" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>315 - SoCal WHP Assessment</t>
         </is>
       </c>
       <c r="H113" s="9" t="inlineStr">
@@ -14309,17 +14317,17 @@
       </c>
       <c r="B114" s="9" t="inlineStr">
         <is>
-          <t>300_UPSERT_INVOICE</t>
+          <t>325_REVIEW_NOTIFICATION</t>
         </is>
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>Upsert Invoice Record (Final/DP)</t>
+          <t>Review Notification (Operations)</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>Runs when a 300 - Account Management record is created or updated, and only if Request Down Payment is 'True' or Submit Final Invoice is 'True'.</t>
+          <t>Runs when a 325 - SoCal Installation record is updated, and only if Installation Status compares to 'None' and Reviewer Name compares to 'None'.</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
@@ -14334,21 +14342,17 @@
       </c>
       <c r="G114" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>325 - SoCal Installation</t>
         </is>
       </c>
       <c r="H114" s="9" t="inlineStr">
         <is>
-          <t>CreateOrUpdate</t>
-        </is>
-      </c>
-      <c r="I114" s="9" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="I114" s="9" t="inlineStr"/>
       <c r="J114" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" ht="22" customHeight="1">
@@ -14359,50 +14363,238 @@
       </c>
       <c r="B115" s="9" t="inlineStr">
         <is>
+          <t>INVOICE_REVIEW_NOTIFICATION</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>Review Notification (Operations)</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) compares to 'None' and Processor Name (Final) compares to 'None' and Invoice Status (Final) is at least 'Pending Review'.</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>WFEngine</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G115" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="H115" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="I115" s="9" t="inlineStr"/>
+      <c r="J115" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B116" s="9" t="inlineStr">
+        <is>
+          <t>300_CONTRACTOR_SUBMITS_3</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>Contractor Submits Assessment Invoice</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>Runs when a 300 - Account Management record is updated, and only if Invoice Assessment is 'True' and Assessment Invoice Amount compares to 'None'.</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>WFEngine</t>
+        </is>
+      </c>
+      <c r="F116" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G116" s="9" t="inlineStr">
+        <is>
+          <t>300 - Account Management</t>
+        </is>
+      </c>
+      <c r="H116" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="I116" s="9" t="inlineStr"/>
+      <c r="J116" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>INVOICE_FINAL_APPROVED_FOR</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>Final Approved for Payment</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>Runs when a Invoice record is updated, and only if Invoice Status (Final) is 'Approved for Final Payment' and Review Status - Management (Final) is 'Approved'.</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>WFEngine</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G117" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="H117" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="I117" s="9" t="inlineStr"/>
+      <c r="J117" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>300_UPSERT_INVOICE</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>Upsert Invoice Record (Final/DP)</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>Runs when a 300 - Account Management record is created or updated, and only if Request Down Payment is 'True' or Submit Final Invoice is 'True'.</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>WFEngine</t>
+        </is>
+      </c>
+      <c r="F118" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G118" s="9" t="inlineStr">
+        <is>
+          <t>300 - Account Management</t>
+        </is>
+      </c>
+      <c r="H118" s="9" t="inlineStr">
+        <is>
+          <t>CreateOrUpdate</t>
+        </is>
+      </c>
+      <c r="I118" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="J118" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
           <t>300_UPDATE_INSTALLATION</t>
         </is>
       </c>
-      <c r="C115" s="9" t="inlineStr">
+      <c r="C119" s="9" t="inlineStr">
         <is>
           <t>Update Installation Contractor for Form 315</t>
         </is>
       </c>
-      <c r="D115" s="9" t="inlineStr">
+      <c r="D119" s="9" t="inlineStr">
         <is>
           <t>Runs when a 300 - Account Management record is updated, and only if Project Stage is 'Installation' and Installation Status is 'In Progress'.</t>
         </is>
       </c>
-      <c r="E115" s="9" t="inlineStr">
+      <c r="E119" s="9" t="inlineStr">
         <is>
           <t>WFEngine</t>
         </is>
       </c>
-      <c r="F115" s="9" t="inlineStr">
+      <c r="F119" s="9" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G115" s="9" t="inlineStr">
+      <c r="G119" s="9" t="inlineStr">
         <is>
           <t>300 - Account Management</t>
         </is>
       </c>
-      <c r="H115" s="9" t="inlineStr">
+      <c r="H119" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="I115" s="9" t="inlineStr">
+      <c r="I119" s="9" t="inlineStr">
         <is>
           <t>315 - SoCal WHP Assessment</t>
         </is>
       </c>
-      <c r="J115" s="9" t="n">
+      <c r="J119" s="9" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J115"/>
+  <autoFilter ref="A3:J119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15501,7 +15693,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>liwp/ENROLLMENT_DESKTOP_REVIEW, liwp/ENROLLMENT_ENROLLMENT_APPROVED, liwp/ENROLLMENT_ENROLLMENT_REJECTED, liwp/ASSESSMENT_DESKTOP_REVIEW, liwp/ACCOUNT_WORK_ORDER_ISSUED, liwp/ASSESSMENT_APPROVED_ISSUE_WORK, liwp/ASSESSMENT_CORRECTIONS_REQUIRED, liwp/INSTALLATI_DESKTOP_REVIEW, liwp/INSTALLATI_APPROVED, liwp/INSTALLATI_CORRECTIONS_REQUIRED, liwp/SOLAR_DESKTOP_REVIEW, liwp/SOLAR_SPV_APPROVED, liwp/SOLAR_SPV_REJECTED, liwp/INSPECTION_NOTE_ADDED_BY, liwp/INSPECTION_INSPECTION_RESULT, liwp/ENERGY_APPROVED_EMAIL, liwp/ENERGY_WAIVER_APPROVED, liwp/ENROLLMENT_REVIEW_NOTIFICATION, liwp/ASSESSMENT_REVIEW_NOTIFICATION, liwp/ASSESSMENT_REVIEW_NOTIFICATION_2, liwp/INSTALLATI_REVIEW_NOTIFICATION, liwp/INVOICE_REVIEW_NOTIFICATION, liwp/INVOICE_APPROVED_BY, liwp/INVOICE_CORRECTIONS_REQUIRED, liwp/INVOICE_CORRECTIONS, sce-be/210_DESKTOP_REVIEW, sce-be/210_ENROLLMENT_APPROVED, sce-be/210_REQUIRES_CORRECTIONS, sce-be/255_INSTALLATION_DESKTOP, sce-be/255_INSTALLATION, sce-be/255_INSTALLATION_2, sce-be/INVOICE_INVOICE_SUBMITTED_BY, sce-be/INVOICE_APPROVED_BY, sce-be/INVOICE_CORRECTIONS_REQUIRED, sce-be/INVOICE_INVOICE_REJECTED_BY, sce-be/INVOICE_CORRECTIONS_REQUIRED_2, sce-be/210_REVIEW_NOTIFICATION, sce-be/255_REVIEW_NOTIFICATION, sce-be/INVOICE_REVIEW_NOTIFICATION, sdge-whp/410_DESKTOP_REVIEW, sdge-whp/410_ENROLLMENT_APPROVED, sdge-whp/410_ENROLLMENT, sdge-whp/415_DESKTOP_REVIEW, sdge-whp/415_ASSESSMENT_APPROVED, sdge-whp/415_ASSESSMENT_REQUIRES, sdge-whp/425_INSTALLATION_READY, sdge-whp/425_INSTALLATION, sdge-whp/425_INSTALLATION_2, sdge-whp/INVOICE_FINAL_INVOICE, sdge-whp/INVOICE_FINAL_APPROVED_BY, sdge-whp/INVOICE_FINAL_APPROVED_FOR, sdge-whp/ACCOUNT_CONTRACTOR_SUBMITS_2, sdge-whp/ACCOUNT_CUSTOMER_INTEREST, sdge-whp/410_REVIEW_NOTIFICATION, sdge-whp/415_REVIEW_NOTIFICATION, sdge-whp/425_REVIEW_NOTIFICATION, sdge-whp/INVOICE_REVIEW_NOTIFICATION, sdge-whp/ACCOUNT_APPROVED_FOR_INSTALL, socal-whp/310_DESKTOP_REVIEW, socal-whp/310_ENROLLMENT_APPROVED, socal-whp/310_ENROLLMENT, socal-whp/315_DESKTOP_REVIEW, socal-whp/315_APPROVED, socal-whp/315_SUBMISSION_RESULTS, socal-whp/300_CUSTOMER_INTEREST, socal-whp/325_READY_FOR_REVIEW, socal-whp/325_INSTALLATION, socal-whp/395_INSPECTION_RESULT, socal-whp/395_WORK_ORDER_ASSIGNED, socal-whp/300_HANDOFF_TO, socal-whp/300_CONTRACTOR, socal-whp/INVOICE_DP_APPROVED_BY, socal-whp/INVOICE_DP_CORRECTIONS, socal-whp/INVOICE_DP_APPROVED_BY_2, socal-whp/INVOICE_FINAL_INVOICE, socal-whp/INVOICE_FINAL_APPROVED_BY, socal-whp/300_CONTRACTOR_SUBMITS, socal-whp/395_UPDATED_NOTE_TO, socal-whp/395_UPDATED_NOTE_BY, socal-whp/300_CONTRACTOR_SUBMITS_2, socal-whp/300_CONTRACTOR_2, socal-whp/INVOICE_ENROLLMENT_INVOICE, socal-whp/INVOICE_ENROLLMENT_INVOICE_2, socal-whp/INVOICE_ENROLLMENT_INVOICE_3, socal-whp/395_UPDATED_NOTE, socal-whp/395_RE_INSPECTION_STATUS, socal-whp/INVOICE_FINAL_INVOICE_2, socal-whp/INVOICE_DP_INVOICE_REJECTED, socal-whp/INVOICE_FINAL_CORRECTIONS, socal-whp/INVOICE_ENROLLMENT_INVOICE_4, socal-whp/INVOICE_CREATE_CUSTOMER, socal-whp/310_NOTIFY_ELITE_DESERT, socal-whp/300_APPROVED_FOR_INSTALL, socal-whp/310_REVIEW_NOTIFICATION, socal-whp/315_REVIEW_NOTIFICATION, socal-whp/325_REVIEW_NOTIFICATION, socal-whp/INVOICE_REVIEW_NOTIFICATION, socal-whp/300_CONTRACTOR_SUBMITS_3, socal-whp/INVOICE_FINAL_APPROVED_FOR</t>
+          <t>liwp/ENROLLMENT_DESKTOP_REVIEW, liwp/ENROLLMENT_ENROLLMENT_APPROVED, liwp/ENROLLMENT_ENROLLMENT_REJECTED, liwp/ASSESSMENT_DESKTOP_REVIEW, liwp/ACCOUNT_WORK_ORDER_ISSUED, liwp/ASSESSMENT_APPROVED_ISSUE_WORK, liwp/ASSESSMENT_CORRECTIONS_REQUIRED, liwp/INSTALLATI_DESKTOP_REVIEW, liwp/INSTALLATI_APPROVED, liwp/INSTALLATI_CORRECTIONS_REQUIRED, liwp/SOLAR_DESKTOP_REVIEW, liwp/SOLAR_SPV_APPROVED, liwp/SOLAR_SPV_REJECTED, liwp/INSPECTION_NOTE_ADDED_BY, liwp/INSPECTION_INSPECTION_RESULT, liwp/ENERGY_APPROVED_EMAIL, liwp/ENERGY_WAIVER_APPROVED, liwp/ENROLLMENT_REVIEW_NOTIFICATION, liwp/ASSESSMENT_REVIEW_NOTIFICATION, liwp/ASSESSMENT_REVIEW_NOTIFICATION_2, liwp/INSTALLATI_REVIEW_NOTIFICATION, liwp/INVOICE_REVIEW_NOTIFICATION, liwp/INVOICE_APPROVED_BY, liwp/INVOICE_CORRECTIONS_REQUIRED, liwp/INVOICE_CORRECTIONS, sce-be/210_DESKTOP_REVIEW, sce-be/210_REQUIRES_CORRECTIONS, sce-be/255_INSTALLATION_DESKTOP, sce-be/255_INSTALLATION, sce-be/255_INSTALLATION_2, sce-be/INVOICE_INVOICE_SUBMITTED_BY, sce-be/INVOICE_APPROVED_BY, sce-be/INVOICE_CORRECTIONS_REQUIRED, sce-be/INVOICE_INVOICE_REJECTED_BY, sce-be/INVOICE_CORRECTIONS_REQUIRED_2, sce-be/210_REVIEW_NOTIFICATION, sce-be/255_REVIEW_NOTIFICATION, sce-be/INVOICE_REVIEW_NOTIFICATION, sce-be/210_ENROLLMENT_APPROVED, sdge-whp/410_DESKTOP_REVIEW, sdge-whp/410_ENROLLMENT_APPROVED, sdge-whp/410_ENROLLMENT, sdge-whp/415_DESKTOP_REVIEW, sdge-whp/415_ASSESSMENT_APPROVED, sdge-whp/415_ASSESSMENT_REQUIRES, sdge-whp/425_INSTALLATION_READY, sdge-whp/425_INSTALLATION, sdge-whp/425_INSTALLATION_2, sdge-whp/INVOICE_FINAL_INVOICE, sdge-whp/INVOICE_FINAL_APPROVED_BY, sdge-whp/INVOICE_FINAL_APPROVED_FOR, sdge-whp/ACCOUNT_CONTRACTOR_SUBMITS_2, sdge-whp/ACCOUNT_CUSTOMER_INTEREST, sdge-whp/410_REVIEW_NOTIFICATION, sdge-whp/415_REVIEW_NOTIFICATION, sdge-whp/425_REVIEW_NOTIFICATION, sdge-whp/INVOICE_REVIEW_NOTIFICATION, sdge-whp/ACCOUNT_APPROVED_FOR_INSTALL, socal-whp/310_DESKTOP_REVIEW, socal-whp/310_ENROLLMENT_APPROVED, socal-whp/310_ENROLLMENT, socal-whp/315_DESKTOP_REVIEW, socal-whp/315_APPROVED, socal-whp/315_SUBMISSION_RESULTS, socal-whp/300_CUSTOMER_INTEREST, socal-whp/325_READY_FOR_REVIEW, socal-whp/325_INSTALLATION, socal-whp/395_INSPECTION_RESULT, socal-whp/395_WORK_ORDER_ASSIGNED, socal-whp/300_HANDOFF_TO, socal-whp/300_CONTRACTOR, socal-whp/INVOICE_DP_APPROVED_BY, socal-whp/INVOICE_DP_CORRECTIONS, socal-whp/INVOICE_DP_APPROVED_BY_2, socal-whp/INVOICE_FINAL_INVOICE, socal-whp/INVOICE_FINAL_APPROVED_BY, socal-whp/300_CONTRACTOR_SUBMITS, socal-whp/395_UPDATED_NOTE_TO, socal-whp/395_UPDATED_NOTE_BY, socal-whp/300_CONTRACTOR_SUBMITS_2, socal-whp/300_CONTRACTOR_2, socal-whp/INVOICE_ENROLLMENT_INVOICE, socal-whp/INVOICE_ENROLLMENT_INVOICE_2, socal-whp/INVOICE_ENROLLMENT_INVOICE_3, socal-whp/395_UPDATED_NOTE, socal-whp/395_RE_INSPECTION_STATUS, socal-whp/INVOICE_FINAL_INVOICE_2, socal-whp/INVOICE_DP_INVOICE_REJECTED, socal-whp/INVOICE_FINAL_CORRECTIONS, socal-whp/INVOICE_ENROLLMENT_INVOICE_4, socal-whp/INVOICE_CREATE_CUSTOMER, socal-whp/310_NOTIFY_ELITE_DESERT, socal-whp/300_APPROVED_FOR_INSTALL, socal-whp/310_REVIEW_NOTIFICATION, socal-whp/315_REVIEW_NOTIFICATION, socal-whp/325_REVIEW_NOTIFICATION, socal-whp/INVOICE_REVIEW_NOTIFICATION, socal-whp/300_CONTRACTOR_SUBMITS_3, socal-whp/INVOICE_FINAL_APPROVED_FOR</t>
         </is>
       </c>
     </row>
@@ -15512,7 +15704,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
@@ -15521,7 +15713,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>liwp/INSPECTION_NEW_WORK_ORDER, liwp/INSPECTION_WORK_ORDER_ASSIGNED, liwp/INVOICE_INVOICE_SUBMITTED_BY, nve-qar/895_DISPATCH_TO_USER, sce-be/200_CUSTOMER_INTEREST, sce-be/INVOICE_INVOICE_SUBMITTED_BY_2, sdge-whp/ACCOUNT_REFRESH_ACCOUNT</t>
+          <t>liwp/INSPECTION_NEW_WORK_ORDER, liwp/INSPECTION_WORK_ORDER_ASSIGNED, liwp/INVOICE_INVOICE_SUBMITTED_BY, nve-qar/895_DISPATCH_TO_USER, sce-be/200_CUSTOMER_INTEREST, sce-be/INVOICE_INVOICE_SUBMITTED_BY_2, sce-be/210_UPDATE_RECORDS, sce-be/255_UPDATE_RECORDS, sdge-whp/ACCOUNT_REFRESH_ACCOUNT</t>
         </is>
       </c>
     </row>
@@ -15557,7 +15749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -15792,12 +15984,12 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake · Update · [(static/other)]</t>
+          <t>210 - Enrollment &amp; Assessment Form · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -15815,7 +16007,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="G8" s="9" t="n">
@@ -15831,12 +16023,12 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment · Update · [(static/other)]</t>
+          <t>310 - Enrollment Intake · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>410 - WH Enrollment</t>
+          <t>310 - Enrollment Intake</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -15854,7 +16046,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>sdge-whp</t>
+          <t>socal-whp</t>
         </is>
       </c>
       <c r="G9" s="9" t="n">
@@ -15870,12 +16062,12 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment · Update · [(static/other)]</t>
+          <t>410 - WH Enrollment · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>415 - San Diego WHP Assessment</t>
+          <t>410 - WH Enrollment</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -15909,12 +16101,12 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Assessment Intake - Form 02 · Update · [(static/other)]</t>
+          <t>415 - San Diego WHP Assessment · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Assessment Intake - Form 02</t>
+          <t>415 - San Diego WHP Assessment</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -15932,7 +16124,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>liwp</t>
+          <t>sdge-whp</t>
         </is>
       </c>
       <c r="G11" s="9" t="n">
@@ -15948,12 +16140,12 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>210 - Enrollment &amp; Assessment Form · Update · [(static/other)]</t>
+          <t>Assessment Intake - Form 02 · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>210 - Enrollment &amp; Assessment Form</t>
+          <t>Assessment Intake - Form 02</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -15967,15 +16159,15 @@
         </is>
       </c>
       <c r="E12" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>sce-be</t>
+          <t>liwp</t>
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
@@ -16299,17 +16491,17 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Energy Audit · Update · [(static/other)]</t>
+          <t>200 - Account · Create · [(static/other)]</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Energy Audit</t>
+          <t>200 - Account</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -16322,7 +16514,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>liwp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="G21" s="9" t="n">
@@ -16338,17 +16530,17 @@
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Inspections · Create · [(static/other)]</t>
+          <t>Energy Audit · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Inspections</t>
+          <t>Energy Audit</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Create</t>
+          <t>Update</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -16377,7 +16569,7 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Inspections · Update · [(static/other)]</t>
+          <t>Inspections · Create · [(static/other)]</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -16387,7 +16579,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -16416,17 +16608,17 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Invoice · Create · [(static/other)]</t>
+          <t>Inspections · Update · [(static/other)]</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Inspections</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Create</t>
+          <t>Update</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -16439,7 +16631,7 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>liwp, sce-be</t>
+          <t>liwp</t>
         </is>
       </c>
       <c r="G24" s="9" t="n">
@@ -16455,12 +16647,12 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>200 - Account · Create · [(static/other)]</t>
+          <t>Invoice · Create · [(static/other)]</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>200 - Account</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -16474,19 +16666,19 @@
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>sce-be</t>
+          <t>liwp, sce-be</t>
         </is>
       </c>
       <c r="G25" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>Drift</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr"/>
@@ -16494,17 +16686,17 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management · CreateOrUpdate · [(static/other)]</t>
+          <t>210 - Enrollment &amp; Assessment Form · Create · [(static/other)]</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>CreateOrUpdate</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -16517,7 +16709,7 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="G26" s="9" t="n">
@@ -16533,12 +16725,12 @@
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>895 - Installation / Warranty · Create · [(static/other)]</t>
+          <t>255 - BE Installation Form · Create · [(static/other)]</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>895 - Installation / Warranty</t>
+          <t>255 - BE Installation Form</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -16556,7 +16748,7 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>nve-qar</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="G27" s="9" t="n">
@@ -16572,17 +16764,17 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Account Management (00) · Update · [(static/other)]</t>
+          <t>300 - Account Management · CreateOrUpdate · [(static/other)]</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Account Management (00)</t>
+          <t>300 - Account Management</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>CreateOrUpdate</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -16595,7 +16787,7 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>liwp</t>
+          <t>socal-whp</t>
         </is>
       </c>
       <c r="G28" s="9" t="n">
@@ -16611,12 +16803,12 @@
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400) · Create · [(static/other)]</t>
+          <t>895 - Installation / Warranty · Create · [(static/other)]</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Account Management (400)</t>
+          <t>895 - Installation / Warranty</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -16634,7 +16826,7 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>sdge-whp</t>
+          <t>nve-qar</t>
         </is>
       </c>
       <c r="G29" s="9" t="n">
@@ -16647,8 +16839,86 @@
       </c>
       <c r="I29" s="9" t="inlineStr"/>
     </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Account Management (00) · Update · [(static/other)]</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Account Management (00)</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>(static/other)</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>liwp</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Account Management (400) · Create · [(static/other)]</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Account Management (400)</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>(static/other)</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>sdge-whp</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:I29"/>
+  <autoFilter ref="A3:I31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Drop socal-whp individual form re-exports, rebuild all outputs
Adds surgical-update exports for 300/310/315/325/395/399/Invoice to
data/socal-whp/forms/, regenerates all workspace + global outputs and
docs/, and prunes an old snapshot in favor of a fresh one.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/global/cross-workspace-inventory.xlsx
+++ b/output/global/cross-workspace-inventory.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Workspaces" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AllForms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AllWorkflows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="FormNameCollisions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DuplicateFlows" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="WorkflowReuse" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="FormFamilies" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FieldTemplates" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AllForms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AllWorkflows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormNameCollisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DuplicateFlows" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowReuse" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormFamilies" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldTemplates" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$9</definedName>

</xml_diff>